<commit_message>
refactor: pisahkan CSS, JS, dan engine ke file terpisah
- Pindahkan CSS inline dari index.html & home.html ke static/style.css
- Pindahkan JS frontend dari index.html ke static/script.js
- Pindahkan forward_chaining dari app.py ke engine.py
- Buat .gitignore (exclude .venv, __pycache__, *.pyc, .vscode/)
- Hapus file sampah 3.1.0
- generate_dataset.py baca data dari knowledge_base (kurangi duplikasi)
</commit_message>
<xml_diff>
--- a/dataset_vetexpert.xlsx
+++ b/dataset_vetexpert.xlsx
@@ -38,7 +38,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -87,6 +87,18 @@
         <bgColor rgb="00F5F5F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E3F2FD"/>
+        <bgColor rgb="00E3F2FD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3E5F5"/>
+        <bgColor rgb="00F3E5F5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -106,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -145,6 +157,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -517,7 +541,7 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -652,7 +676,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Toxoplasmosis</t>
+          <t>Feline Panleukopenia</t>
         </is>
       </c>
     </row>
@@ -669,7 +693,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Toxoplasmosis</t>
+          <t>Canine Parvovirus</t>
         </is>
       </c>
     </row>
@@ -686,7 +710,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Toxoplasmosis</t>
+          <t>Canine Parvovirus</t>
         </is>
       </c>
     </row>
@@ -703,7 +727,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Toxoplasmosis</t>
+          <t>Canine Parvovirus</t>
         </is>
       </c>
     </row>
@@ -720,7 +744,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Toxoplasmosis</t>
+          <t>Canine Parvovirus</t>
         </is>
       </c>
     </row>
@@ -754,7 +778,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Toxoplasmosis</t>
+          <t>Feline Panleukopenia</t>
         </is>
       </c>
     </row>
@@ -771,7 +795,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Toxoplasmosis</t>
+          <t>Feline Panleukopenia</t>
         </is>
       </c>
     </row>
@@ -907,7 +931,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Rabies</t>
+          <t>Canine Parvovirus</t>
         </is>
       </c>
     </row>
@@ -956,7 +980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1306,7 +1330,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>G01, G05, G15, G17</t>
+          <t>G05, G06, G15, G17</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -1351,6 +1375,122 @@
       </c>
       <c r="G13" s="4" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>R13</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>G07, G08</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Gejala ringan Feline Panleukopenia</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>R14</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>G07, G08, G11, G13, G14</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Gejala berat Feline Panleukopenia</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>R15</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>G08, G09</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Gejala ringan Canine Parvovirus</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>R16</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>G08, G09, G10, G11, G22</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Gejala berat Canine Parvovirus</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1364,7 +1504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1789,7 +1929,7 @@
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>G05, G15, G17</t>
+          <t>G05, G06, G15, G17</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr">
@@ -1830,6 +1970,146 @@
       <c r="G13" s="13" t="inlineStr">
         <is>
           <t>G01, G02, G03, G04</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>R13</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>Feline Panleukopenia</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>Kucing</t>
+        </is>
+      </c>
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>G07, G08</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>G01, G02, G03</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>D14</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>R14</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>Feline Panleukopenia</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>Kucing</t>
+        </is>
+      </c>
+      <c r="F15" s="15" t="inlineStr">
+        <is>
+          <t>G07, G08, G11, G13, G14</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>G01, G02, G03</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>D15</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>R15</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>Canine Parvovirus</t>
+        </is>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>Anjing</t>
+        </is>
+      </c>
+      <c r="F16" s="17" t="inlineStr">
+        <is>
+          <t>G08, G09</t>
+        </is>
+      </c>
+      <c r="G16" s="17" t="inlineStr">
+        <is>
+          <t>G01, G02, G03</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>D16</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>R16</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>Canine Parvovirus</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>Anjing</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="inlineStr">
+        <is>
+          <t>G08, G09, G10, G11, G22</t>
+        </is>
+      </c>
+      <c r="G17" s="17" t="inlineStr">
+        <is>
+          <t>G01, G02, G03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: hapus FP/CPV, bersihkan dead code, tambah logo & link Halodoc
- Hapus P03/P04 dari knowledge_base.py (kembali ke 2 penyakit)
- Hapus dead code PENYAKIT_RULES & GRUP di index.html
- Hapus unused import GEJALA di test_dataset.py
- Hapus aturan FP/CPV dari generate_dataset.py
- Tambah favicon SVG + route /favicon.ico redirect
- Tambah validasi POST body (non-JSON → 400)
- Tambah logo di navbar (home + diagnosa)
- Tambah button "Konsultasi via Halodoc" di panel diagnosa
</commit_message>
<xml_diff>
--- a/dataset_vetexpert.xlsx
+++ b/dataset_vetexpert.xlsx
@@ -38,7 +38,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -87,18 +87,6 @@
         <bgColor rgb="00F5F5F5"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E3F2FD"/>
-        <bgColor rgb="00E3F2FD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F3E5F5"/>
-        <bgColor rgb="00F3E5F5"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -118,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -157,18 +145,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -676,7 +652,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Feline Panleukopenia</t>
+          <t>Toxoplasmosis</t>
         </is>
       </c>
     </row>
@@ -693,7 +669,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Canine Parvovirus</t>
+          <t>Toxoplasmosis</t>
         </is>
       </c>
     </row>
@@ -710,7 +686,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Canine Parvovirus</t>
+          <t>Toxoplasmosis</t>
         </is>
       </c>
     </row>
@@ -727,7 +703,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Canine Parvovirus</t>
+          <t>Toxoplasmosis</t>
         </is>
       </c>
     </row>
@@ -744,7 +720,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Canine Parvovirus</t>
+          <t>Toxoplasmosis</t>
         </is>
       </c>
     </row>
@@ -778,7 +754,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Feline Panleukopenia</t>
+          <t>Toxoplasmosis</t>
         </is>
       </c>
     </row>
@@ -795,7 +771,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Feline Panleukopenia</t>
+          <t>Toxoplasmosis</t>
         </is>
       </c>
     </row>
@@ -931,7 +907,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Canine Parvovirus</t>
+          <t>Rabies</t>
         </is>
       </c>
     </row>
@@ -980,7 +956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1377,122 +1353,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>R13</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>G07, G08</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Gejala ringan Feline Panleukopenia</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>R14</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>G07, G08, G11, G13, G14</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Gejala berat Feline Panleukopenia</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="4" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>R15</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>G08, G09</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>Gejala ringan Canine Parvovirus</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>R16</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>G08, G09, G10, G11, G22</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Gejala berat Canine Parvovirus</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="F17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>2</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1504,7 +1364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1973,146 +1833,6 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="14" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="14" t="inlineStr">
-        <is>
-          <t>D13</t>
-        </is>
-      </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>R13</t>
-        </is>
-      </c>
-      <c r="D14" s="15" t="inlineStr">
-        <is>
-          <t>Feline Panleukopenia</t>
-        </is>
-      </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>Kucing</t>
-        </is>
-      </c>
-      <c r="F14" s="15" t="inlineStr">
-        <is>
-          <t>G07, G08</t>
-        </is>
-      </c>
-      <c r="G14" s="15" t="inlineStr">
-        <is>
-          <t>G01, G02, G03</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="14" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="14" t="inlineStr">
-        <is>
-          <t>D14</t>
-        </is>
-      </c>
-      <c r="C15" s="14" t="inlineStr">
-        <is>
-          <t>R14</t>
-        </is>
-      </c>
-      <c r="D15" s="15" t="inlineStr">
-        <is>
-          <t>Feline Panleukopenia</t>
-        </is>
-      </c>
-      <c r="E15" s="14" t="inlineStr">
-        <is>
-          <t>Kucing</t>
-        </is>
-      </c>
-      <c r="F15" s="15" t="inlineStr">
-        <is>
-          <t>G07, G08, G11, G13, G14</t>
-        </is>
-      </c>
-      <c r="G15" s="15" t="inlineStr">
-        <is>
-          <t>G01, G02, G03</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="16" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="16" t="inlineStr">
-        <is>
-          <t>D15</t>
-        </is>
-      </c>
-      <c r="C16" s="16" t="inlineStr">
-        <is>
-          <t>R15</t>
-        </is>
-      </c>
-      <c r="D16" s="17" t="inlineStr">
-        <is>
-          <t>Canine Parvovirus</t>
-        </is>
-      </c>
-      <c r="E16" s="16" t="inlineStr">
-        <is>
-          <t>Anjing</t>
-        </is>
-      </c>
-      <c r="F16" s="17" t="inlineStr">
-        <is>
-          <t>G08, G09</t>
-        </is>
-      </c>
-      <c r="G16" s="17" t="inlineStr">
-        <is>
-          <t>G01, G02, G03</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="16" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="16" t="inlineStr">
-        <is>
-          <t>D16</t>
-        </is>
-      </c>
-      <c r="C17" s="16" t="inlineStr">
-        <is>
-          <t>R16</t>
-        </is>
-      </c>
-      <c r="D17" s="17" t="inlineStr">
-        <is>
-          <t>Canine Parvovirus</t>
-        </is>
-      </c>
-      <c r="E17" s="16" t="inlineStr">
-        <is>
-          <t>Anjing</t>
-        </is>
-      </c>
-      <c r="F17" s="17" t="inlineStr">
-        <is>
-          <t>G08, G09, G10, G11, G22</t>
-        </is>
-      </c>
-      <c r="G17" s="17" t="inlineStr">
-        <is>
-          <t>G01, G02, G03</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>